<commit_message>
Preserve dashboard text selection during live refresh
</commit_message>
<xml_diff>
--- a/input/containers.xlsx
+++ b/input/containers.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuxiaolong/Documents/Projects/container_tracker/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA795C58-04B4-EA44-8939-40469FD148F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA540168-E62E-2E49-B710-EC9D5457B5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="33880" yWindow="2780" windowWidth="19240" windowHeight="29480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1902" uniqueCount="912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="1013">
   <si>
     <t>Container</t>
   </si>
@@ -2761,6 +2761,310 @@
   </si>
   <si>
     <t>ZCSU6921790</t>
+  </si>
+  <si>
+    <t>EITU8141328</t>
+  </si>
+  <si>
+    <t>TGBU6509109</t>
+  </si>
+  <si>
+    <t>MAGU5380377</t>
+  </si>
+  <si>
+    <t>TCLU6329898</t>
+  </si>
+  <si>
+    <t>EITU9740995</t>
+  </si>
+  <si>
+    <t>EGSU9773522</t>
+  </si>
+  <si>
+    <t>EMCU8806577</t>
+  </si>
+  <si>
+    <t>TRHU8127109</t>
+  </si>
+  <si>
+    <t>EGSU1947510</t>
+  </si>
+  <si>
+    <t>EGSU6318649</t>
+  </si>
+  <si>
+    <t>TXGU5590736</t>
+  </si>
+  <si>
+    <t>TIIU5227389</t>
+  </si>
+  <si>
+    <t>EMCU0164378</t>
+  </si>
+  <si>
+    <t>EGSU6516201</t>
+  </si>
+  <si>
+    <t>TGBU7294577</t>
+  </si>
+  <si>
+    <t>EGSU9352647</t>
+  </si>
+  <si>
+    <t>EGSU0250304</t>
+  </si>
+  <si>
+    <t>EGSU0058550</t>
+  </si>
+  <si>
+    <t>EITU9558635</t>
+  </si>
+  <si>
+    <t>EGHU9473096</t>
+  </si>
+  <si>
+    <t>TRHU7145263</t>
+  </si>
+  <si>
+    <t>EGSU0391149</t>
+  </si>
+  <si>
+    <t>GCXU6262947</t>
+  </si>
+  <si>
+    <t>EMCU8893864</t>
+  </si>
+  <si>
+    <t>EMCU8367330</t>
+  </si>
+  <si>
+    <t>EMCU8737603</t>
+  </si>
+  <si>
+    <t>CAAU5870764</t>
+  </si>
+  <si>
+    <t>CAAU5562210</t>
+  </si>
+  <si>
+    <t>TXGU5757844</t>
+  </si>
+  <si>
+    <t>EGSU9492778</t>
+  </si>
+  <si>
+    <t>EMCU8578040</t>
+  </si>
+  <si>
+    <t>EGSU9240462</t>
+  </si>
+  <si>
+    <t>EMCU0095214</t>
+  </si>
+  <si>
+    <t>EGHU8390612</t>
+  </si>
+  <si>
+    <t>EMCU1842058</t>
+  </si>
+  <si>
+    <t>EGSU6418817</t>
+  </si>
+  <si>
+    <t>EITU1962471</t>
+  </si>
+  <si>
+    <t>EITU1880455</t>
+  </si>
+  <si>
+    <t>EGSU6358359</t>
+  </si>
+  <si>
+    <t>EMCU5980163</t>
+  </si>
+  <si>
+    <t>TRHU7757490</t>
+  </si>
+  <si>
+    <t>TXGU5842740</t>
+  </si>
+  <si>
+    <t>EGSU6009866</t>
+  </si>
+  <si>
+    <t>EITU9137554</t>
+  </si>
+  <si>
+    <t>EGSU0251764</t>
+  </si>
+  <si>
+    <t>EGSU6593888</t>
+  </si>
+  <si>
+    <t>EGHU9179224</t>
+  </si>
+  <si>
+    <t>TXGU8187160</t>
+  </si>
+  <si>
+    <t>EITU1985923</t>
+  </si>
+  <si>
+    <t>EGSU0309212</t>
+  </si>
+  <si>
+    <t>EMCU0094244</t>
+  </si>
+  <si>
+    <t>EITU9253425</t>
+  </si>
+  <si>
+    <t>GAOU6287352</t>
+  </si>
+  <si>
+    <t>EMCU8267665</t>
+  </si>
+  <si>
+    <t>EMCU8266226</t>
+  </si>
+  <si>
+    <t>TRHU6277820</t>
+  </si>
+  <si>
+    <t>EGSU6266890</t>
+  </si>
+  <si>
+    <t>FFAU5163446</t>
+  </si>
+  <si>
+    <t>TCLU6332628</t>
+  </si>
+  <si>
+    <t>TRHU7502972</t>
+  </si>
+  <si>
+    <t>EGSU6096433</t>
+  </si>
+  <si>
+    <t>EGSU0051262</t>
+  </si>
+  <si>
+    <t>EITU9787035</t>
+  </si>
+  <si>
+    <t>EMCU1511050</t>
+  </si>
+  <si>
+    <t>TGBU9973108</t>
+  </si>
+  <si>
+    <t>EITU9763012</t>
+  </si>
+  <si>
+    <t>EGSU6427188</t>
+  </si>
+  <si>
+    <t>EGSU6067219</t>
+  </si>
+  <si>
+    <t>CAAU6004907</t>
+  </si>
+  <si>
+    <t>TRHU5826904</t>
+  </si>
+  <si>
+    <t>EGSU0337385</t>
+  </si>
+  <si>
+    <t>TXGU5852477</t>
+  </si>
+  <si>
+    <t>EITU8124254</t>
+  </si>
+  <si>
+    <t>TXGU6090627</t>
+  </si>
+  <si>
+    <t>TIIU6040258</t>
+  </si>
+  <si>
+    <t>EMCU8510939</t>
+  </si>
+  <si>
+    <t>TXGU5614057</t>
+  </si>
+  <si>
+    <t>DFSU6999920</t>
+  </si>
+  <si>
+    <t>EGSU6741352</t>
+  </si>
+  <si>
+    <t>EGHU8362550</t>
+  </si>
+  <si>
+    <t>EMCU0129680</t>
+  </si>
+  <si>
+    <t>TXGU6805192</t>
+  </si>
+  <si>
+    <t>EGSU1268437</t>
+  </si>
+  <si>
+    <t>EGSU0366444</t>
+  </si>
+  <si>
+    <t>TXGU5582812</t>
+  </si>
+  <si>
+    <t>TRHU6545877</t>
+  </si>
+  <si>
+    <t>EMCU8673089</t>
+  </si>
+  <si>
+    <t>GAOU6922442</t>
+  </si>
+  <si>
+    <t>EGSU6741687</t>
+  </si>
+  <si>
+    <t>TCKU6052321</t>
+  </si>
+  <si>
+    <t>TIIU6496525</t>
+  </si>
+  <si>
+    <t>DRYU9908178</t>
+  </si>
+  <si>
+    <t>EGSU1498018</t>
+  </si>
+  <si>
+    <t>TXGU5306310</t>
+  </si>
+  <si>
+    <t>TGBU6723810</t>
+  </si>
+  <si>
+    <t>FFAU1597737</t>
+  </si>
+  <si>
+    <t>EGSU1769510</t>
+  </si>
+  <si>
+    <t>TXGU7802480</t>
+  </si>
+  <si>
+    <t>EMCU8779297</t>
+  </si>
+  <si>
+    <t>EGSU6536614</t>
+  </si>
+  <si>
+    <t>EGLV</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -3124,7 +3428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B949"/>
+  <dimension ref="A1:B1049"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -10721,6 +11025,806 @@
       </c>
       <c r="B949" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="950" spans="1:2">
+      <c r="A950" t="s">
+        <v>912</v>
+      </c>
+      <c r="B950" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="951" spans="1:2">
+      <c r="A951" t="s">
+        <v>913</v>
+      </c>
+      <c r="B951" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="952" spans="1:2">
+      <c r="A952" t="s">
+        <v>914</v>
+      </c>
+      <c r="B952" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="953" spans="1:2">
+      <c r="A953" t="s">
+        <v>915</v>
+      </c>
+      <c r="B953" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="954" spans="1:2">
+      <c r="A954" t="s">
+        <v>916</v>
+      </c>
+      <c r="B954" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="955" spans="1:2">
+      <c r="A955" t="s">
+        <v>917</v>
+      </c>
+      <c r="B955" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="956" spans="1:2">
+      <c r="A956" t="s">
+        <v>918</v>
+      </c>
+      <c r="B956" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="957" spans="1:2">
+      <c r="A957" t="s">
+        <v>919</v>
+      </c>
+      <c r="B957" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="958" spans="1:2">
+      <c r="A958" t="s">
+        <v>920</v>
+      </c>
+      <c r="B958" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="959" spans="1:2">
+      <c r="A959" t="s">
+        <v>921</v>
+      </c>
+      <c r="B959" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="960" spans="1:2">
+      <c r="A960" t="s">
+        <v>922</v>
+      </c>
+      <c r="B960" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="961" spans="1:2">
+      <c r="A961" t="s">
+        <v>923</v>
+      </c>
+      <c r="B961" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="962" spans="1:2">
+      <c r="A962" t="s">
+        <v>924</v>
+      </c>
+      <c r="B962" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="963" spans="1:2">
+      <c r="A963" t="s">
+        <v>925</v>
+      </c>
+      <c r="B963" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="964" spans="1:2">
+      <c r="A964" t="s">
+        <v>926</v>
+      </c>
+      <c r="B964" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="965" spans="1:2">
+      <c r="A965" t="s">
+        <v>927</v>
+      </c>
+      <c r="B965" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="966" spans="1:2">
+      <c r="A966" t="s">
+        <v>928</v>
+      </c>
+      <c r="B966" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="967" spans="1:2">
+      <c r="A967" t="s">
+        <v>929</v>
+      </c>
+      <c r="B967" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="968" spans="1:2">
+      <c r="A968" t="s">
+        <v>930</v>
+      </c>
+      <c r="B968" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="969" spans="1:2">
+      <c r="A969" t="s">
+        <v>931</v>
+      </c>
+      <c r="B969" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="970" spans="1:2">
+      <c r="A970" t="s">
+        <v>932</v>
+      </c>
+      <c r="B970" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="971" spans="1:2">
+      <c r="A971" t="s">
+        <v>933</v>
+      </c>
+      <c r="B971" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="972" spans="1:2">
+      <c r="A972" t="s">
+        <v>934</v>
+      </c>
+      <c r="B972" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="973" spans="1:2">
+      <c r="A973" t="s">
+        <v>935</v>
+      </c>
+      <c r="B973" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="974" spans="1:2">
+      <c r="A974" t="s">
+        <v>936</v>
+      </c>
+      <c r="B974" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="975" spans="1:2">
+      <c r="A975" t="s">
+        <v>937</v>
+      </c>
+      <c r="B975" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="976" spans="1:2">
+      <c r="A976" t="s">
+        <v>938</v>
+      </c>
+      <c r="B976" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="977" spans="1:2">
+      <c r="A977" t="s">
+        <v>939</v>
+      </c>
+      <c r="B977" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="978" spans="1:2">
+      <c r="A978" t="s">
+        <v>940</v>
+      </c>
+      <c r="B978" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="979" spans="1:2">
+      <c r="A979" t="s">
+        <v>941</v>
+      </c>
+      <c r="B979" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="980" spans="1:2">
+      <c r="A980" t="s">
+        <v>942</v>
+      </c>
+      <c r="B980" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="981" spans="1:2">
+      <c r="A981" t="s">
+        <v>943</v>
+      </c>
+      <c r="B981" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="982" spans="1:2">
+      <c r="A982" t="s">
+        <v>944</v>
+      </c>
+      <c r="B982" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="983" spans="1:2">
+      <c r="A983" t="s">
+        <v>945</v>
+      </c>
+      <c r="B983" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="984" spans="1:2">
+      <c r="A984" t="s">
+        <v>946</v>
+      </c>
+      <c r="B984" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="985" spans="1:2">
+      <c r="A985" t="s">
+        <v>947</v>
+      </c>
+      <c r="B985" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="986" spans="1:2">
+      <c r="A986" t="s">
+        <v>948</v>
+      </c>
+      <c r="B986" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="987" spans="1:2">
+      <c r="A987" t="s">
+        <v>949</v>
+      </c>
+      <c r="B987" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="988" spans="1:2">
+      <c r="A988" t="s">
+        <v>950</v>
+      </c>
+      <c r="B988" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="989" spans="1:2">
+      <c r="A989" t="s">
+        <v>951</v>
+      </c>
+      <c r="B989" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="990" spans="1:2">
+      <c r="A990" t="s">
+        <v>952</v>
+      </c>
+      <c r="B990" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="991" spans="1:2">
+      <c r="A991" t="s">
+        <v>953</v>
+      </c>
+      <c r="B991" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="992" spans="1:2">
+      <c r="A992" t="s">
+        <v>954</v>
+      </c>
+      <c r="B992" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="993" spans="1:2">
+      <c r="A993" t="s">
+        <v>955</v>
+      </c>
+      <c r="B993" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="994" spans="1:2">
+      <c r="A994" t="s">
+        <v>956</v>
+      </c>
+      <c r="B994" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="995" spans="1:2">
+      <c r="A995" t="s">
+        <v>957</v>
+      </c>
+      <c r="B995" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="996" spans="1:2">
+      <c r="A996" t="s">
+        <v>958</v>
+      </c>
+      <c r="B996" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="997" spans="1:2">
+      <c r="A997" t="s">
+        <v>959</v>
+      </c>
+      <c r="B997" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="998" spans="1:2">
+      <c r="A998" t="s">
+        <v>960</v>
+      </c>
+      <c r="B998" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="999" spans="1:2">
+      <c r="A999" t="s">
+        <v>961</v>
+      </c>
+      <c r="B999" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1000" spans="1:2">
+      <c r="A1000" t="s">
+        <v>962</v>
+      </c>
+      <c r="B1000" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1001" spans="1:2">
+      <c r="A1001" t="s">
+        <v>963</v>
+      </c>
+      <c r="B1001" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1002" spans="1:2">
+      <c r="A1002" t="s">
+        <v>964</v>
+      </c>
+      <c r="B1002" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1003" spans="1:2">
+      <c r="A1003" t="s">
+        <v>965</v>
+      </c>
+      <c r="B1003" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1004" spans="1:2">
+      <c r="A1004" t="s">
+        <v>966</v>
+      </c>
+      <c r="B1004" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1005" spans="1:2">
+      <c r="A1005" t="s">
+        <v>967</v>
+      </c>
+      <c r="B1005" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1006" spans="1:2">
+      <c r="A1006" t="s">
+        <v>968</v>
+      </c>
+      <c r="B1006" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1007" spans="1:2">
+      <c r="A1007" t="s">
+        <v>969</v>
+      </c>
+      <c r="B1007" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:2">
+      <c r="A1008" t="s">
+        <v>970</v>
+      </c>
+      <c r="B1008" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:2">
+      <c r="A1009" t="s">
+        <v>971</v>
+      </c>
+      <c r="B1009" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:2">
+      <c r="A1010" t="s">
+        <v>972</v>
+      </c>
+      <c r="B1010" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:2">
+      <c r="A1011" t="s">
+        <v>973</v>
+      </c>
+      <c r="B1011" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:2">
+      <c r="A1012" t="s">
+        <v>974</v>
+      </c>
+      <c r="B1012" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:2">
+      <c r="A1013" t="s">
+        <v>975</v>
+      </c>
+      <c r="B1013" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:2">
+      <c r="A1014" t="s">
+        <v>976</v>
+      </c>
+      <c r="B1014" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:2">
+      <c r="A1015" t="s">
+        <v>977</v>
+      </c>
+      <c r="B1015" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:2">
+      <c r="A1016" t="s">
+        <v>978</v>
+      </c>
+      <c r="B1016" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:2">
+      <c r="A1017" t="s">
+        <v>979</v>
+      </c>
+      <c r="B1017" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:2">
+      <c r="A1018" t="s">
+        <v>980</v>
+      </c>
+      <c r="B1018" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:2">
+      <c r="A1019" t="s">
+        <v>981</v>
+      </c>
+      <c r="B1019" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:2">
+      <c r="A1020" t="s">
+        <v>982</v>
+      </c>
+      <c r="B1020" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:2">
+      <c r="A1021" t="s">
+        <v>983</v>
+      </c>
+      <c r="B1021" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:2">
+      <c r="A1022" t="s">
+        <v>984</v>
+      </c>
+      <c r="B1022" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:2">
+      <c r="A1023" t="s">
+        <v>985</v>
+      </c>
+      <c r="B1023" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:2">
+      <c r="A1024" t="s">
+        <v>986</v>
+      </c>
+      <c r="B1024" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:2">
+      <c r="A1025" t="s">
+        <v>987</v>
+      </c>
+      <c r="B1025" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:2">
+      <c r="A1026" t="s">
+        <v>988</v>
+      </c>
+      <c r="B1026" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:2">
+      <c r="A1027" t="s">
+        <v>989</v>
+      </c>
+      <c r="B1027" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:2">
+      <c r="A1028" t="s">
+        <v>990</v>
+      </c>
+      <c r="B1028" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:2">
+      <c r="A1029" t="s">
+        <v>991</v>
+      </c>
+      <c r="B1029" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:2">
+      <c r="A1030" t="s">
+        <v>992</v>
+      </c>
+      <c r="B1030" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:2">
+      <c r="A1031" t="s">
+        <v>993</v>
+      </c>
+      <c r="B1031" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1032" spans="1:2">
+      <c r="A1032" t="s">
+        <v>994</v>
+      </c>
+      <c r="B1032" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:2">
+      <c r="A1033" t="s">
+        <v>995</v>
+      </c>
+      <c r="B1033" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:2">
+      <c r="A1034" t="s">
+        <v>996</v>
+      </c>
+      <c r="B1034" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:2">
+      <c r="A1035" t="s">
+        <v>997</v>
+      </c>
+      <c r="B1035" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1036" spans="1:2">
+      <c r="A1036" t="s">
+        <v>998</v>
+      </c>
+      <c r="B1036" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:2">
+      <c r="A1037" t="s">
+        <v>999</v>
+      </c>
+      <c r="B1037" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:2">
+      <c r="A1038" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B1038" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:2">
+      <c r="A1039" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B1039" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1040" spans="1:2">
+      <c r="A1040" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B1040" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:2">
+      <c r="A1041" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B1041" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:2">
+      <c r="A1042" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B1042" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:2">
+      <c r="A1043" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B1043" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:2">
+      <c r="A1044" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B1044" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:2">
+      <c r="A1045" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B1045" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:2">
+      <c r="A1046" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B1046" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1047" spans="1:2">
+      <c r="A1047" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B1047" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1048" spans="1:2">
+      <c r="A1048" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B1048" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="1049" spans="1:2">
+      <c r="A1049" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B1049" t="s">
+        <v>1012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>